<commit_message>
Comprehensive push of other changes.
</commit_message>
<xml_diff>
--- a/data/template/SOC Evaluation Template - 2024.xlsx
+++ b/data/template/SOC Evaluation Template - 2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nandps-my.sharepoint.com/personal/brian_klumpp_solidigmtechnology_com/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nandps-my.sharepoint.com/personal/brian_klumpp_solidigmtechnology_com/Documents/Documents/Python Scripts/SOCAnalyzer5/data/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{6B34E3CB-9927-4D1B-AF95-7033E03B8FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{598150F9-8E80-4A6A-9A12-84289217380E}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="8_{6B34E3CB-9927-4D1B-AF95-7033E03B8FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{964AEC2A-EAB1-4834-9439-3745754E6AB9}"/>
   <bookViews>
-    <workbookView xWindow="-93" yWindow="-93" windowWidth="27493" windowHeight="13866" tabRatio="888" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="27493" windowHeight="13866" tabRatio="888" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Basic Procedures" sheetId="1" r:id="rId1"/>
@@ -959,6 +959,10 @@
     <xf numFmtId="15" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -969,15 +973,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1039,14 +1043,10 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1282,6 +1282,9 @@
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
   <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
         <we:customFunctionIds>_xldudf_AI_TABLE</we:customFunctionIds>
@@ -1418,11 +1421,11 @@
       <c r="W4" s="4"/>
     </row>
     <row r="5" spans="1:23" ht="12.7" x14ac:dyDescent="0.4">
-      <c r="A5" s="68" t="s">
+      <c r="A5" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="69"/>
-      <c r="C5" s="69"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="71"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
@@ -1846,9 +1849,9 @@
       <c r="W20" s="4"/>
     </row>
     <row r="21" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="70"/>
-      <c r="B21" s="69"/>
-      <c r="C21" s="69"/>
+      <c r="A21" s="72"/>
+      <c r="B21" s="71"/>
+      <c r="C21" s="71"/>
       <c r="D21" s="19"/>
       <c r="E21" s="19"/>
       <c r="F21" s="19"/>
@@ -1871,9 +1874,9 @@
       <c r="W21" s="19"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="71"/>
-      <c r="B22" s="69"/>
-      <c r="C22" s="69"/>
+      <c r="A22" s="73"/>
+      <c r="B22" s="71"/>
+      <c r="C22" s="71"/>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
       <c r="F22" s="19"/>
@@ -14466,7 +14469,7 @@
       <c r="T6" s="33"/>
     </row>
     <row r="7" spans="1:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="77" t="s">
         <v>33</v>
       </c>
       <c r="B7" s="74" t="s">
@@ -14474,7 +14477,7 @@
       </c>
       <c r="C7" s="75"/>
       <c r="D7" s="76"/>
-      <c r="E7" s="102"/>
+      <c r="E7" s="68"/>
       <c r="F7" s="33"/>
       <c r="G7" s="33"/>
       <c r="H7" s="33"/>
@@ -14492,7 +14495,7 @@
       <c r="T7" s="33"/>
     </row>
     <row r="8" spans="1:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="72"/>
+      <c r="A8" s="78"/>
       <c r="B8" s="62" t="s">
         <v>35</v>
       </c>
@@ -14502,7 +14505,7 @@
       <c r="D8" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="103" t="s">
+      <c r="E8" s="69" t="s">
         <v>72</v>
       </c>
       <c r="F8" s="33"/>
@@ -19744,7 +19747,7 @@
       <c r="R4" s="35"/>
     </row>
     <row r="5" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="77" t="s">
+      <c r="A5" s="79" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="75"/>
@@ -19786,10 +19789,10 @@
       <c r="R6" s="35"/>
     </row>
     <row r="7" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="78" t="s">
+      <c r="A7" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="69"/>
+      <c r="B7" s="71"/>
       <c r="C7" s="35"/>
       <c r="D7" s="33"/>
       <c r="E7" s="33"/>
@@ -22978,7 +22981,7 @@
       <c r="V4" s="35"/>
     </row>
     <row r="5" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="77" t="s">
+      <c r="A5" s="79" t="s">
         <v>47</v>
       </c>
       <c r="B5" s="75"/>
@@ -46431,7 +46434,7 @@
       <c r="R4" s="35"/>
     </row>
     <row r="5" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="79" t="s">
+      <c r="A5" s="81" t="s">
         <v>51</v>
       </c>
       <c r="B5" s="75"/>
@@ -46473,7 +46476,7 @@
       <c r="R6" s="35"/>
     </row>
     <row r="7" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="80" t="s">
+      <c r="A7" s="82" t="s">
         <v>52</v>
       </c>
       <c r="B7" s="75"/>
@@ -46611,7 +46614,7 @@
       <c r="AB11" s="33"/>
     </row>
     <row r="12" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="80" t="s">
+      <c r="A12" s="82" t="s">
         <v>59</v>
       </c>
       <c r="B12" s="75"/>
@@ -49665,13 +49668,13 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="81" t="s">
+      <c r="B10" s="83" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="82"/>
-      <c r="D10" s="82"/>
-      <c r="E10" s="82"/>
-      <c r="F10" s="83"/>
+      <c r="C10" s="84"/>
+      <c r="D10" s="84"/>
+      <c r="E10" s="84"/>
+      <c r="F10" s="85"/>
     </row>
     <row r="11" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="12" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.4"/>
@@ -50748,11 +50751,11 @@
     </row>
     <row r="5" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="35"/>
-      <c r="B5" s="84" t="s">
+      <c r="B5" s="86" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="69"/>
-      <c r="D5" s="69"/>
+      <c r="C5" s="71"/>
+      <c r="D5" s="71"/>
       <c r="E5" s="35"/>
       <c r="F5" s="35"/>
       <c r="G5" s="35"/>
@@ -50764,13 +50767,13 @@
     </row>
     <row r="6" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="35"/>
-      <c r="B6" s="85" t="s">
+      <c r="B6" s="87" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="86"/>
-      <c r="D6" s="86"/>
-      <c r="E6" s="86"/>
-      <c r="F6" s="87"/>
+      <c r="C6" s="88"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="89"/>
       <c r="G6" s="35"/>
       <c r="H6" s="35"/>
       <c r="I6" s="35"/>
@@ -50780,11 +50783,11 @@
     </row>
     <row r="7" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="35"/>
-      <c r="B7" s="88"/>
-      <c r="C7" s="69"/>
-      <c r="D7" s="69"/>
-      <c r="E7" s="69"/>
-      <c r="F7" s="89"/>
+      <c r="B7" s="90"/>
+      <c r="C7" s="71"/>
+      <c r="D7" s="71"/>
+      <c r="E7" s="71"/>
+      <c r="F7" s="91"/>
       <c r="G7" s="35"/>
       <c r="H7" s="35"/>
       <c r="I7" s="35"/>
@@ -50794,11 +50797,11 @@
     </row>
     <row r="8" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="35"/>
-      <c r="B8" s="88"/>
-      <c r="C8" s="69"/>
-      <c r="D8" s="69"/>
-      <c r="E8" s="69"/>
-      <c r="F8" s="89"/>
+      <c r="B8" s="90"/>
+      <c r="C8" s="71"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="91"/>
       <c r="G8" s="35"/>
       <c r="H8" s="35"/>
       <c r="I8" s="35"/>
@@ -50808,11 +50811,11 @@
     </row>
     <row r="9" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="35"/>
-      <c r="B9" s="90"/>
-      <c r="C9" s="91"/>
-      <c r="D9" s="91"/>
-      <c r="E9" s="91"/>
-      <c r="F9" s="92"/>
+      <c r="B9" s="92"/>
+      <c r="C9" s="93"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="94"/>
       <c r="G9" s="35"/>
       <c r="H9" s="35"/>
       <c r="I9" s="35"/>
@@ -50867,408 +50870,408 @@
     </row>
     <row r="13" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="35"/>
-      <c r="B13" s="93"/>
-      <c r="C13" s="94"/>
-      <c r="D13" s="94"/>
-      <c r="E13" s="94"/>
-      <c r="F13" s="94"/>
-      <c r="G13" s="94"/>
-      <c r="H13" s="94"/>
-      <c r="I13" s="94"/>
-      <c r="J13" s="94"/>
-      <c r="K13" s="94"/>
-      <c r="L13" s="94"/>
-      <c r="M13" s="95"/>
+      <c r="B13" s="95"/>
+      <c r="C13" s="96"/>
+      <c r="D13" s="96"/>
+      <c r="E13" s="96"/>
+      <c r="F13" s="96"/>
+      <c r="G13" s="96"/>
+      <c r="H13" s="96"/>
+      <c r="I13" s="96"/>
+      <c r="J13" s="96"/>
+      <c r="K13" s="96"/>
+      <c r="L13" s="96"/>
+      <c r="M13" s="97"/>
     </row>
     <row r="14" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="35"/>
-      <c r="B14" s="96"/>
-      <c r="C14" s="97"/>
-      <c r="D14" s="97"/>
-      <c r="E14" s="97"/>
-      <c r="F14" s="97"/>
-      <c r="G14" s="97"/>
-      <c r="H14" s="97"/>
-      <c r="I14" s="97"/>
-      <c r="J14" s="97"/>
-      <c r="K14" s="97"/>
-      <c r="L14" s="97"/>
-      <c r="M14" s="98"/>
+      <c r="B14" s="98"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="99"/>
+      <c r="F14" s="99"/>
+      <c r="G14" s="99"/>
+      <c r="H14" s="99"/>
+      <c r="I14" s="99"/>
+      <c r="J14" s="99"/>
+      <c r="K14" s="99"/>
+      <c r="L14" s="99"/>
+      <c r="M14" s="100"/>
     </row>
     <row r="15" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="35"/>
-      <c r="B15" s="96"/>
-      <c r="C15" s="97"/>
-      <c r="D15" s="97"/>
-      <c r="E15" s="97"/>
-      <c r="F15" s="97"/>
-      <c r="G15" s="97"/>
-      <c r="H15" s="97"/>
-      <c r="I15" s="97"/>
-      <c r="J15" s="97"/>
-      <c r="K15" s="97"/>
-      <c r="L15" s="97"/>
-      <c r="M15" s="98"/>
+      <c r="B15" s="98"/>
+      <c r="C15" s="99"/>
+      <c r="D15" s="99"/>
+      <c r="E15" s="99"/>
+      <c r="F15" s="99"/>
+      <c r="G15" s="99"/>
+      <c r="H15" s="99"/>
+      <c r="I15" s="99"/>
+      <c r="J15" s="99"/>
+      <c r="K15" s="99"/>
+      <c r="L15" s="99"/>
+      <c r="M15" s="100"/>
     </row>
     <row r="16" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="35"/>
-      <c r="B16" s="96"/>
-      <c r="C16" s="97"/>
-      <c r="D16" s="97"/>
-      <c r="E16" s="97"/>
-      <c r="F16" s="97"/>
-      <c r="G16" s="97"/>
-      <c r="H16" s="97"/>
-      <c r="I16" s="97"/>
-      <c r="J16" s="97"/>
-      <c r="K16" s="97"/>
-      <c r="L16" s="97"/>
-      <c r="M16" s="98"/>
+      <c r="B16" s="98"/>
+      <c r="C16" s="99"/>
+      <c r="D16" s="99"/>
+      <c r="E16" s="99"/>
+      <c r="F16" s="99"/>
+      <c r="G16" s="99"/>
+      <c r="H16" s="99"/>
+      <c r="I16" s="99"/>
+      <c r="J16" s="99"/>
+      <c r="K16" s="99"/>
+      <c r="L16" s="99"/>
+      <c r="M16" s="100"/>
     </row>
     <row r="17" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="35"/>
-      <c r="B17" s="96"/>
-      <c r="C17" s="97"/>
-      <c r="D17" s="97"/>
-      <c r="E17" s="97"/>
-      <c r="F17" s="97"/>
-      <c r="G17" s="97"/>
-      <c r="H17" s="97"/>
-      <c r="I17" s="97"/>
-      <c r="J17" s="97"/>
-      <c r="K17" s="97"/>
-      <c r="L17" s="97"/>
-      <c r="M17" s="98"/>
+      <c r="B17" s="98"/>
+      <c r="C17" s="99"/>
+      <c r="D17" s="99"/>
+      <c r="E17" s="99"/>
+      <c r="F17" s="99"/>
+      <c r="G17" s="99"/>
+      <c r="H17" s="99"/>
+      <c r="I17" s="99"/>
+      <c r="J17" s="99"/>
+      <c r="K17" s="99"/>
+      <c r="L17" s="99"/>
+      <c r="M17" s="100"/>
     </row>
     <row r="18" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="35"/>
-      <c r="B18" s="96"/>
-      <c r="C18" s="97"/>
-      <c r="D18" s="97"/>
-      <c r="E18" s="97"/>
-      <c r="F18" s="97"/>
-      <c r="G18" s="97"/>
-      <c r="H18" s="97"/>
-      <c r="I18" s="97"/>
-      <c r="J18" s="97"/>
-      <c r="K18" s="97"/>
-      <c r="L18" s="97"/>
-      <c r="M18" s="98"/>
+      <c r="B18" s="98"/>
+      <c r="C18" s="99"/>
+      <c r="D18" s="99"/>
+      <c r="E18" s="99"/>
+      <c r="F18" s="99"/>
+      <c r="G18" s="99"/>
+      <c r="H18" s="99"/>
+      <c r="I18" s="99"/>
+      <c r="J18" s="99"/>
+      <c r="K18" s="99"/>
+      <c r="L18" s="99"/>
+      <c r="M18" s="100"/>
     </row>
     <row r="19" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="35"/>
-      <c r="B19" s="96"/>
-      <c r="C19" s="97"/>
-      <c r="D19" s="97"/>
-      <c r="E19" s="97"/>
-      <c r="F19" s="97"/>
-      <c r="G19" s="97"/>
-      <c r="H19" s="97"/>
-      <c r="I19" s="97"/>
-      <c r="J19" s="97"/>
-      <c r="K19" s="97"/>
-      <c r="L19" s="97"/>
-      <c r="M19" s="98"/>
+      <c r="B19" s="98"/>
+      <c r="C19" s="99"/>
+      <c r="D19" s="99"/>
+      <c r="E19" s="99"/>
+      <c r="F19" s="99"/>
+      <c r="G19" s="99"/>
+      <c r="H19" s="99"/>
+      <c r="I19" s="99"/>
+      <c r="J19" s="99"/>
+      <c r="K19" s="99"/>
+      <c r="L19" s="99"/>
+      <c r="M19" s="100"/>
     </row>
     <row r="20" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="35"/>
-      <c r="B20" s="96"/>
-      <c r="C20" s="97"/>
-      <c r="D20" s="97"/>
-      <c r="E20" s="97"/>
-      <c r="F20" s="97"/>
-      <c r="G20" s="97"/>
-      <c r="H20" s="97"/>
-      <c r="I20" s="97"/>
-      <c r="J20" s="97"/>
-      <c r="K20" s="97"/>
-      <c r="L20" s="97"/>
-      <c r="M20" s="98"/>
+      <c r="B20" s="98"/>
+      <c r="C20" s="99"/>
+      <c r="D20" s="99"/>
+      <c r="E20" s="99"/>
+      <c r="F20" s="99"/>
+      <c r="G20" s="99"/>
+      <c r="H20" s="99"/>
+      <c r="I20" s="99"/>
+      <c r="J20" s="99"/>
+      <c r="K20" s="99"/>
+      <c r="L20" s="99"/>
+      <c r="M20" s="100"/>
     </row>
     <row r="21" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="35"/>
-      <c r="B21" s="96"/>
-      <c r="C21" s="97"/>
-      <c r="D21" s="97"/>
-      <c r="E21" s="97"/>
-      <c r="F21" s="97"/>
-      <c r="G21" s="97"/>
-      <c r="H21" s="97"/>
-      <c r="I21" s="97"/>
-      <c r="J21" s="97"/>
-      <c r="K21" s="97"/>
-      <c r="L21" s="97"/>
-      <c r="M21" s="98"/>
+      <c r="B21" s="98"/>
+      <c r="C21" s="99"/>
+      <c r="D21" s="99"/>
+      <c r="E21" s="99"/>
+      <c r="F21" s="99"/>
+      <c r="G21" s="99"/>
+      <c r="H21" s="99"/>
+      <c r="I21" s="99"/>
+      <c r="J21" s="99"/>
+      <c r="K21" s="99"/>
+      <c r="L21" s="99"/>
+      <c r="M21" s="100"/>
     </row>
     <row r="22" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="35"/>
-      <c r="B22" s="96"/>
-      <c r="C22" s="97"/>
-      <c r="D22" s="97"/>
-      <c r="E22" s="97"/>
-      <c r="F22" s="97"/>
-      <c r="G22" s="97"/>
-      <c r="H22" s="97"/>
-      <c r="I22" s="97"/>
-      <c r="J22" s="97"/>
-      <c r="K22" s="97"/>
-      <c r="L22" s="97"/>
-      <c r="M22" s="98"/>
+      <c r="B22" s="98"/>
+      <c r="C22" s="99"/>
+      <c r="D22" s="99"/>
+      <c r="E22" s="99"/>
+      <c r="F22" s="99"/>
+      <c r="G22" s="99"/>
+      <c r="H22" s="99"/>
+      <c r="I22" s="99"/>
+      <c r="J22" s="99"/>
+      <c r="K22" s="99"/>
+      <c r="L22" s="99"/>
+      <c r="M22" s="100"/>
     </row>
     <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="35"/>
-      <c r="B23" s="96"/>
-      <c r="C23" s="97"/>
-      <c r="D23" s="97"/>
-      <c r="E23" s="97"/>
-      <c r="F23" s="97"/>
-      <c r="G23" s="97"/>
-      <c r="H23" s="97"/>
-      <c r="I23" s="97"/>
-      <c r="J23" s="97"/>
-      <c r="K23" s="97"/>
-      <c r="L23" s="97"/>
-      <c r="M23" s="98"/>
+      <c r="B23" s="98"/>
+      <c r="C23" s="99"/>
+      <c r="D23" s="99"/>
+      <c r="E23" s="99"/>
+      <c r="F23" s="99"/>
+      <c r="G23" s="99"/>
+      <c r="H23" s="99"/>
+      <c r="I23" s="99"/>
+      <c r="J23" s="99"/>
+      <c r="K23" s="99"/>
+      <c r="L23" s="99"/>
+      <c r="M23" s="100"/>
     </row>
     <row r="24" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="35"/>
-      <c r="B24" s="96"/>
-      <c r="C24" s="97"/>
-      <c r="D24" s="97"/>
-      <c r="E24" s="97"/>
-      <c r="F24" s="97"/>
-      <c r="G24" s="97"/>
-      <c r="H24" s="97"/>
-      <c r="I24" s="97"/>
-      <c r="J24" s="97"/>
-      <c r="K24" s="97"/>
-      <c r="L24" s="97"/>
-      <c r="M24" s="98"/>
+      <c r="B24" s="98"/>
+      <c r="C24" s="99"/>
+      <c r="D24" s="99"/>
+      <c r="E24" s="99"/>
+      <c r="F24" s="99"/>
+      <c r="G24" s="99"/>
+      <c r="H24" s="99"/>
+      <c r="I24" s="99"/>
+      <c r="J24" s="99"/>
+      <c r="K24" s="99"/>
+      <c r="L24" s="99"/>
+      <c r="M24" s="100"/>
     </row>
     <row r="25" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="35"/>
-      <c r="B25" s="96"/>
-      <c r="C25" s="97"/>
-      <c r="D25" s="97"/>
-      <c r="E25" s="97"/>
-      <c r="F25" s="97"/>
-      <c r="G25" s="97"/>
-      <c r="H25" s="97"/>
-      <c r="I25" s="97"/>
-      <c r="J25" s="97"/>
-      <c r="K25" s="97"/>
-      <c r="L25" s="97"/>
-      <c r="M25" s="98"/>
+      <c r="B25" s="98"/>
+      <c r="C25" s="99"/>
+      <c r="D25" s="99"/>
+      <c r="E25" s="99"/>
+      <c r="F25" s="99"/>
+      <c r="G25" s="99"/>
+      <c r="H25" s="99"/>
+      <c r="I25" s="99"/>
+      <c r="J25" s="99"/>
+      <c r="K25" s="99"/>
+      <c r="L25" s="99"/>
+      <c r="M25" s="100"/>
     </row>
     <row r="26" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="35"/>
-      <c r="B26" s="96"/>
-      <c r="C26" s="97"/>
-      <c r="D26" s="97"/>
-      <c r="E26" s="97"/>
-      <c r="F26" s="97"/>
-      <c r="G26" s="97"/>
-      <c r="H26" s="97"/>
-      <c r="I26" s="97"/>
-      <c r="J26" s="97"/>
-      <c r="K26" s="97"/>
-      <c r="L26" s="97"/>
-      <c r="M26" s="98"/>
+      <c r="B26" s="98"/>
+      <c r="C26" s="99"/>
+      <c r="D26" s="99"/>
+      <c r="E26" s="99"/>
+      <c r="F26" s="99"/>
+      <c r="G26" s="99"/>
+      <c r="H26" s="99"/>
+      <c r="I26" s="99"/>
+      <c r="J26" s="99"/>
+      <c r="K26" s="99"/>
+      <c r="L26" s="99"/>
+      <c r="M26" s="100"/>
     </row>
     <row r="27" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="35"/>
-      <c r="B27" s="96"/>
-      <c r="C27" s="97"/>
-      <c r="D27" s="97"/>
-      <c r="E27" s="97"/>
-      <c r="F27" s="97"/>
-      <c r="G27" s="97"/>
-      <c r="H27" s="97"/>
-      <c r="I27" s="97"/>
-      <c r="J27" s="97"/>
-      <c r="K27" s="97"/>
-      <c r="L27" s="97"/>
-      <c r="M27" s="98"/>
+      <c r="B27" s="98"/>
+      <c r="C27" s="99"/>
+      <c r="D27" s="99"/>
+      <c r="E27" s="99"/>
+      <c r="F27" s="99"/>
+      <c r="G27" s="99"/>
+      <c r="H27" s="99"/>
+      <c r="I27" s="99"/>
+      <c r="J27" s="99"/>
+      <c r="K27" s="99"/>
+      <c r="L27" s="99"/>
+      <c r="M27" s="100"/>
     </row>
     <row r="28" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="35"/>
-      <c r="B28" s="96"/>
-      <c r="C28" s="97"/>
-      <c r="D28" s="97"/>
-      <c r="E28" s="97"/>
-      <c r="F28" s="97"/>
-      <c r="G28" s="97"/>
-      <c r="H28" s="97"/>
-      <c r="I28" s="97"/>
-      <c r="J28" s="97"/>
-      <c r="K28" s="97"/>
-      <c r="L28" s="97"/>
-      <c r="M28" s="98"/>
+      <c r="B28" s="98"/>
+      <c r="C28" s="99"/>
+      <c r="D28" s="99"/>
+      <c r="E28" s="99"/>
+      <c r="F28" s="99"/>
+      <c r="G28" s="99"/>
+      <c r="H28" s="99"/>
+      <c r="I28" s="99"/>
+      <c r="J28" s="99"/>
+      <c r="K28" s="99"/>
+      <c r="L28" s="99"/>
+      <c r="M28" s="100"/>
     </row>
     <row r="29" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="35"/>
-      <c r="B29" s="96"/>
-      <c r="C29" s="97"/>
-      <c r="D29" s="97"/>
-      <c r="E29" s="97"/>
-      <c r="F29" s="97"/>
-      <c r="G29" s="97"/>
-      <c r="H29" s="97"/>
-      <c r="I29" s="97"/>
-      <c r="J29" s="97"/>
-      <c r="K29" s="97"/>
-      <c r="L29" s="97"/>
-      <c r="M29" s="98"/>
+      <c r="B29" s="98"/>
+      <c r="C29" s="99"/>
+      <c r="D29" s="99"/>
+      <c r="E29" s="99"/>
+      <c r="F29" s="99"/>
+      <c r="G29" s="99"/>
+      <c r="H29" s="99"/>
+      <c r="I29" s="99"/>
+      <c r="J29" s="99"/>
+      <c r="K29" s="99"/>
+      <c r="L29" s="99"/>
+      <c r="M29" s="100"/>
     </row>
     <row r="30" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="35"/>
-      <c r="B30" s="96"/>
-      <c r="C30" s="97"/>
-      <c r="D30" s="97"/>
-      <c r="E30" s="97"/>
-      <c r="F30" s="97"/>
-      <c r="G30" s="97"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="97"/>
-      <c r="J30" s="97"/>
-      <c r="K30" s="97"/>
-      <c r="L30" s="97"/>
-      <c r="M30" s="98"/>
+      <c r="B30" s="98"/>
+      <c r="C30" s="99"/>
+      <c r="D30" s="99"/>
+      <c r="E30" s="99"/>
+      <c r="F30" s="99"/>
+      <c r="G30" s="99"/>
+      <c r="H30" s="99"/>
+      <c r="I30" s="99"/>
+      <c r="J30" s="99"/>
+      <c r="K30" s="99"/>
+      <c r="L30" s="99"/>
+      <c r="M30" s="100"/>
     </row>
     <row r="31" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="35"/>
-      <c r="B31" s="96"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="97"/>
-      <c r="E31" s="97"/>
-      <c r="F31" s="97"/>
-      <c r="G31" s="97"/>
-      <c r="H31" s="97"/>
-      <c r="I31" s="97"/>
-      <c r="J31" s="97"/>
-      <c r="K31" s="97"/>
-      <c r="L31" s="97"/>
-      <c r="M31" s="98"/>
+      <c r="B31" s="98"/>
+      <c r="C31" s="99"/>
+      <c r="D31" s="99"/>
+      <c r="E31" s="99"/>
+      <c r="F31" s="99"/>
+      <c r="G31" s="99"/>
+      <c r="H31" s="99"/>
+      <c r="I31" s="99"/>
+      <c r="J31" s="99"/>
+      <c r="K31" s="99"/>
+      <c r="L31" s="99"/>
+      <c r="M31" s="100"/>
     </row>
     <row r="32" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="35"/>
-      <c r="B32" s="96"/>
-      <c r="C32" s="97"/>
-      <c r="D32" s="97"/>
-      <c r="E32" s="97"/>
-      <c r="F32" s="97"/>
-      <c r="G32" s="97"/>
-      <c r="H32" s="97"/>
-      <c r="I32" s="97"/>
-      <c r="J32" s="97"/>
-      <c r="K32" s="97"/>
-      <c r="L32" s="97"/>
-      <c r="M32" s="98"/>
+      <c r="B32" s="98"/>
+      <c r="C32" s="99"/>
+      <c r="D32" s="99"/>
+      <c r="E32" s="99"/>
+      <c r="F32" s="99"/>
+      <c r="G32" s="99"/>
+      <c r="H32" s="99"/>
+      <c r="I32" s="99"/>
+      <c r="J32" s="99"/>
+      <c r="K32" s="99"/>
+      <c r="L32" s="99"/>
+      <c r="M32" s="100"/>
     </row>
     <row r="33" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="35"/>
-      <c r="B33" s="96"/>
-      <c r="C33" s="97"/>
-      <c r="D33" s="97"/>
-      <c r="E33" s="97"/>
-      <c r="F33" s="97"/>
-      <c r="G33" s="97"/>
-      <c r="H33" s="97"/>
-      <c r="I33" s="97"/>
-      <c r="J33" s="97"/>
-      <c r="K33" s="97"/>
-      <c r="L33" s="97"/>
-      <c r="M33" s="98"/>
+      <c r="B33" s="98"/>
+      <c r="C33" s="99"/>
+      <c r="D33" s="99"/>
+      <c r="E33" s="99"/>
+      <c r="F33" s="99"/>
+      <c r="G33" s="99"/>
+      <c r="H33" s="99"/>
+      <c r="I33" s="99"/>
+      <c r="J33" s="99"/>
+      <c r="K33" s="99"/>
+      <c r="L33" s="99"/>
+      <c r="M33" s="100"/>
     </row>
     <row r="34" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="35"/>
-      <c r="B34" s="96"/>
-      <c r="C34" s="97"/>
-      <c r="D34" s="97"/>
-      <c r="E34" s="97"/>
-      <c r="F34" s="97"/>
-      <c r="G34" s="97"/>
-      <c r="H34" s="97"/>
-      <c r="I34" s="97"/>
-      <c r="J34" s="97"/>
-      <c r="K34" s="97"/>
-      <c r="L34" s="97"/>
-      <c r="M34" s="98"/>
+      <c r="B34" s="98"/>
+      <c r="C34" s="99"/>
+      <c r="D34" s="99"/>
+      <c r="E34" s="99"/>
+      <c r="F34" s="99"/>
+      <c r="G34" s="99"/>
+      <c r="H34" s="99"/>
+      <c r="I34" s="99"/>
+      <c r="J34" s="99"/>
+      <c r="K34" s="99"/>
+      <c r="L34" s="99"/>
+      <c r="M34" s="100"/>
     </row>
     <row r="35" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="35"/>
-      <c r="B35" s="96"/>
-      <c r="C35" s="97"/>
-      <c r="D35" s="97"/>
-      <c r="E35" s="97"/>
-      <c r="F35" s="97"/>
-      <c r="G35" s="97"/>
-      <c r="H35" s="97"/>
-      <c r="I35" s="97"/>
-      <c r="J35" s="97"/>
-      <c r="K35" s="97"/>
-      <c r="L35" s="97"/>
-      <c r="M35" s="98"/>
+      <c r="B35" s="98"/>
+      <c r="C35" s="99"/>
+      <c r="D35" s="99"/>
+      <c r="E35" s="99"/>
+      <c r="F35" s="99"/>
+      <c r="G35" s="99"/>
+      <c r="H35" s="99"/>
+      <c r="I35" s="99"/>
+      <c r="J35" s="99"/>
+      <c r="K35" s="99"/>
+      <c r="L35" s="99"/>
+      <c r="M35" s="100"/>
     </row>
     <row r="36" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="35"/>
-      <c r="B36" s="96"/>
-      <c r="C36" s="97"/>
-      <c r="D36" s="97"/>
-      <c r="E36" s="97"/>
-      <c r="F36" s="97"/>
-      <c r="G36" s="97"/>
-      <c r="H36" s="97"/>
-      <c r="I36" s="97"/>
-      <c r="J36" s="97"/>
-      <c r="K36" s="97"/>
-      <c r="L36" s="97"/>
-      <c r="M36" s="98"/>
+      <c r="B36" s="98"/>
+      <c r="C36" s="99"/>
+      <c r="D36" s="99"/>
+      <c r="E36" s="99"/>
+      <c r="F36" s="99"/>
+      <c r="G36" s="99"/>
+      <c r="H36" s="99"/>
+      <c r="I36" s="99"/>
+      <c r="J36" s="99"/>
+      <c r="K36" s="99"/>
+      <c r="L36" s="99"/>
+      <c r="M36" s="100"/>
     </row>
     <row r="37" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="35"/>
-      <c r="B37" s="96"/>
-      <c r="C37" s="97"/>
-      <c r="D37" s="97"/>
-      <c r="E37" s="97"/>
-      <c r="F37" s="97"/>
-      <c r="G37" s="97"/>
-      <c r="H37" s="97"/>
-      <c r="I37" s="97"/>
-      <c r="J37" s="97"/>
-      <c r="K37" s="97"/>
-      <c r="L37" s="97"/>
-      <c r="M37" s="98"/>
+      <c r="B37" s="98"/>
+      <c r="C37" s="99"/>
+      <c r="D37" s="99"/>
+      <c r="E37" s="99"/>
+      <c r="F37" s="99"/>
+      <c r="G37" s="99"/>
+      <c r="H37" s="99"/>
+      <c r="I37" s="99"/>
+      <c r="J37" s="99"/>
+      <c r="K37" s="99"/>
+      <c r="L37" s="99"/>
+      <c r="M37" s="100"/>
     </row>
     <row r="38" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="35"/>
-      <c r="B38" s="96"/>
-      <c r="C38" s="97"/>
-      <c r="D38" s="97"/>
-      <c r="E38" s="97"/>
-      <c r="F38" s="97"/>
-      <c r="G38" s="97"/>
-      <c r="H38" s="97"/>
-      <c r="I38" s="97"/>
-      <c r="J38" s="97"/>
-      <c r="K38" s="97"/>
-      <c r="L38" s="97"/>
-      <c r="M38" s="98"/>
+      <c r="B38" s="98"/>
+      <c r="C38" s="99"/>
+      <c r="D38" s="99"/>
+      <c r="E38" s="99"/>
+      <c r="F38" s="99"/>
+      <c r="G38" s="99"/>
+      <c r="H38" s="99"/>
+      <c r="I38" s="99"/>
+      <c r="J38" s="99"/>
+      <c r="K38" s="99"/>
+      <c r="L38" s="99"/>
+      <c r="M38" s="100"/>
     </row>
     <row r="39" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="35"/>
-      <c r="B39" s="99"/>
-      <c r="C39" s="100"/>
-      <c r="D39" s="100"/>
-      <c r="E39" s="100"/>
-      <c r="F39" s="100"/>
-      <c r="G39" s="100"/>
-      <c r="H39" s="100"/>
-      <c r="I39" s="100"/>
-      <c r="J39" s="100"/>
-      <c r="K39" s="100"/>
-      <c r="L39" s="100"/>
-      <c r="M39" s="101"/>
+      <c r="B39" s="101"/>
+      <c r="C39" s="102"/>
+      <c r="D39" s="102"/>
+      <c r="E39" s="102"/>
+      <c r="F39" s="102"/>
+      <c r="G39" s="102"/>
+      <c r="H39" s="102"/>
+      <c r="I39" s="102"/>
+      <c r="J39" s="102"/>
+      <c r="K39" s="102"/>
+      <c r="L39" s="102"/>
+      <c r="M39" s="103"/>
     </row>
     <row r="40" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="35"/>
@@ -53296,6 +53299,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EDE5E0A92B1B4245AFCBD746CEDF4560" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6025169be789cc966a04e918ccf67bd3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="7c036ba9-6adb-4bb7-998f-df2d2059af4e" xmlns:ns3="90750662-e876-4027-87c5-760b0ce6cf5c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9a948267c2c89e6701a2eb25cc5d1211" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -53541,15 +53553,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -53564,6 +53567,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0A3F0B4-9A99-4E66-9809-E917735194F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3442C85-1F30-471D-8C30-03DE269E8971}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -53579,14 +53590,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0A3F0B4-9A99-4E66-9809-E917735194F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
chore: Update Excel template
</commit_message>
<xml_diff>
--- a/data/template/SOC Evaluation Template - 2024.xlsx
+++ b/data/template/SOC Evaluation Template - 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nandps-my.sharepoint.com/personal/brian_klumpp_solidigmtechnology_com/Documents/Documents/Python Scripts/SOCAnalyzer5/data/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{6B34E3CB-9927-4D1B-AF95-7033E03B8FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{964AEC2A-EAB1-4834-9439-3745754E6AB9}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{6B34E3CB-9927-4D1B-AF95-7033E03B8FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38484900-A9D4-40CA-B65B-3757BCFC959B}"/>
   <bookViews>
-    <workbookView xWindow="-93" yWindow="-93" windowWidth="27493" windowHeight="13866" tabRatio="888" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="27493" windowHeight="13866" tabRatio="888" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Basic Procedures" sheetId="1" r:id="rId1"/>
@@ -963,6 +963,12 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1042,12 +1048,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1421,11 +1421,11 @@
       <c r="W4" s="4"/>
     </row>
     <row r="5" spans="1:23" ht="12.7" x14ac:dyDescent="0.4">
-      <c r="A5" s="70" t="s">
+      <c r="A5" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="71"/>
-      <c r="C5" s="71"/>
+      <c r="B5" s="73"/>
+      <c r="C5" s="73"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
@@ -1849,9 +1849,9 @@
       <c r="W20" s="4"/>
     </row>
     <row r="21" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="72"/>
-      <c r="B21" s="71"/>
-      <c r="C21" s="71"/>
+      <c r="A21" s="74"/>
+      <c r="B21" s="73"/>
+      <c r="C21" s="73"/>
       <c r="D21" s="19"/>
       <c r="E21" s="19"/>
       <c r="F21" s="19"/>
@@ -1874,9 +1874,9 @@
       <c r="W21" s="19"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="73"/>
-      <c r="B22" s="71"/>
-      <c r="C22" s="71"/>
+      <c r="A22" s="75"/>
+      <c r="B22" s="73"/>
+      <c r="C22" s="73"/>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
       <c r="F22" s="19"/>
@@ -14469,14 +14469,14 @@
       <c r="T6" s="33"/>
     </row>
     <row r="7" spans="1:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="77" t="s">
+      <c r="A7" s="79" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="B7" s="76" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="75"/>
-      <c r="D7" s="76"/>
+      <c r="C7" s="77"/>
+      <c r="D7" s="78"/>
       <c r="E7" s="68"/>
       <c r="F7" s="33"/>
       <c r="G7" s="33"/>
@@ -14495,7 +14495,7 @@
       <c r="T7" s="33"/>
     </row>
     <row r="8" spans="1:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="78"/>
+      <c r="A8" s="80"/>
       <c r="B8" s="62" t="s">
         <v>35</v>
       </c>
@@ -19747,16 +19747,16 @@
       <c r="R4" s="35"/>
     </row>
     <row r="5" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="79" t="s">
+      <c r="A5" s="81" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
-      <c r="G5" s="75"/>
-      <c r="H5" s="76"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="78"/>
       <c r="I5" s="35"/>
       <c r="J5" s="35"/>
       <c r="K5" s="35"/>
@@ -19789,10 +19789,10 @@
       <c r="R6" s="35"/>
     </row>
     <row r="7" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="80" t="s">
+      <c r="A7" s="82" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="71"/>
+      <c r="B7" s="73"/>
       <c r="C7" s="35"/>
       <c r="D7" s="33"/>
       <c r="E7" s="33"/>
@@ -22981,13 +22981,13 @@
       <c r="V4" s="35"/>
     </row>
     <row r="5" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="79" t="s">
+      <c r="A5" s="81" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="77"/>
       <c r="F5" s="35"/>
       <c r="G5" s="35"/>
       <c r="H5" s="35"/>
@@ -46434,13 +46434,13 @@
       <c r="R4" s="35"/>
     </row>
     <row r="5" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="81" t="s">
+      <c r="A5" s="83" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="76"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="78"/>
       <c r="F5" s="35"/>
       <c r="G5" s="35"/>
       <c r="H5" s="35"/>
@@ -46476,16 +46476,16 @@
       <c r="R6" s="35"/>
     </row>
     <row r="7" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="82" t="s">
+      <c r="A7" s="84" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
-      <c r="E7" s="75"/>
-      <c r="F7" s="75"/>
-      <c r="G7" s="75"/>
-      <c r="H7" s="76"/>
+      <c r="B7" s="77"/>
+      <c r="C7" s="77"/>
+      <c r="D7" s="77"/>
+      <c r="E7" s="77"/>
+      <c r="F7" s="77"/>
+      <c r="G7" s="77"/>
+      <c r="H7" s="78"/>
       <c r="I7" s="35"/>
       <c r="J7" s="47"/>
       <c r="K7" s="35"/>
@@ -46534,14 +46534,14 @@
       <c r="R8" s="35"/>
     </row>
     <row r="9" spans="1:28" ht="12.7" x14ac:dyDescent="0.4">
-      <c r="A9" s="104"/>
-      <c r="B9" s="104"/>
-      <c r="C9" s="105"/>
-      <c r="D9" s="104"/>
-      <c r="E9" s="104"/>
-      <c r="F9" s="105"/>
-      <c r="G9" s="105"/>
-      <c r="H9" s="105"/>
+      <c r="A9" s="70"/>
+      <c r="B9" s="70"/>
+      <c r="C9" s="71"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="71"/>
+      <c r="G9" s="71"/>
+      <c r="H9" s="71"/>
       <c r="I9" s="35"/>
       <c r="J9" s="35"/>
       <c r="K9" s="35"/>
@@ -46614,13 +46614,13 @@
       <c r="AB11" s="33"/>
     </row>
     <row r="12" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="82" t="s">
+      <c r="A12" s="84" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="75"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="75"/>
-      <c r="E12" s="76"/>
+      <c r="B12" s="77"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="77"/>
+      <c r="E12" s="78"/>
       <c r="F12" s="35"/>
       <c r="G12" s="35"/>
       <c r="H12" s="35"/>
@@ -49668,13 +49668,13 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="83" t="s">
+      <c r="B10" s="85" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="84"/>
-      <c r="D10" s="84"/>
-      <c r="E10" s="84"/>
-      <c r="F10" s="85"/>
+      <c r="C10" s="86"/>
+      <c r="D10" s="86"/>
+      <c r="E10" s="86"/>
+      <c r="F10" s="87"/>
     </row>
     <row r="11" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="12" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.4"/>
@@ -50751,11 +50751,11 @@
     </row>
     <row r="5" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="35"/>
-      <c r="B5" s="86" t="s">
+      <c r="B5" s="88" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
       <c r="E5" s="35"/>
       <c r="F5" s="35"/>
       <c r="G5" s="35"/>
@@ -50767,13 +50767,13 @@
     </row>
     <row r="6" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="35"/>
-      <c r="B6" s="87" t="s">
+      <c r="B6" s="89" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="88"/>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="89"/>
+      <c r="C6" s="90"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="91"/>
       <c r="G6" s="35"/>
       <c r="H6" s="35"/>
       <c r="I6" s="35"/>
@@ -50783,11 +50783,11 @@
     </row>
     <row r="7" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="35"/>
-      <c r="B7" s="90"/>
-      <c r="C7" s="71"/>
-      <c r="D7" s="71"/>
-      <c r="E7" s="71"/>
-      <c r="F7" s="91"/>
+      <c r="B7" s="92"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="73"/>
+      <c r="E7" s="73"/>
+      <c r="F7" s="93"/>
       <c r="G7" s="35"/>
       <c r="H7" s="35"/>
       <c r="I7" s="35"/>
@@ -50797,11 +50797,11 @@
     </row>
     <row r="8" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="35"/>
-      <c r="B8" s="90"/>
-      <c r="C8" s="71"/>
-      <c r="D8" s="71"/>
-      <c r="E8" s="71"/>
-      <c r="F8" s="91"/>
+      <c r="B8" s="92"/>
+      <c r="C8" s="73"/>
+      <c r="D8" s="73"/>
+      <c r="E8" s="73"/>
+      <c r="F8" s="93"/>
       <c r="G8" s="35"/>
       <c r="H8" s="35"/>
       <c r="I8" s="35"/>
@@ -50811,11 +50811,11 @@
     </row>
     <row r="9" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="35"/>
-      <c r="B9" s="92"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="94"/>
+      <c r="B9" s="94"/>
+      <c r="C9" s="95"/>
+      <c r="D9" s="95"/>
+      <c r="E9" s="95"/>
+      <c r="F9" s="96"/>
       <c r="G9" s="35"/>
       <c r="H9" s="35"/>
       <c r="I9" s="35"/>
@@ -50868,410 +50868,410 @@
       <c r="L12" s="54"/>
       <c r="M12" s="55"/>
     </row>
-    <row r="13" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="35"/>
-      <c r="B13" s="95"/>
-      <c r="C13" s="96"/>
-      <c r="D13" s="96"/>
-      <c r="E13" s="96"/>
-      <c r="F13" s="96"/>
-      <c r="G13" s="96"/>
-      <c r="H13" s="96"/>
-      <c r="I13" s="96"/>
-      <c r="J13" s="96"/>
-      <c r="K13" s="96"/>
-      <c r="L13" s="96"/>
-      <c r="M13" s="97"/>
-    </row>
-    <row r="14" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B13" s="97"/>
+      <c r="C13" s="98"/>
+      <c r="D13" s="98"/>
+      <c r="E13" s="98"/>
+      <c r="F13" s="98"/>
+      <c r="G13" s="98"/>
+      <c r="H13" s="98"/>
+      <c r="I13" s="98"/>
+      <c r="J13" s="98"/>
+      <c r="K13" s="98"/>
+      <c r="L13" s="98"/>
+      <c r="M13" s="99"/>
+    </row>
+    <row r="14" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="35"/>
-      <c r="B14" s="98"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="99"/>
-      <c r="F14" s="99"/>
-      <c r="G14" s="99"/>
-      <c r="H14" s="99"/>
-      <c r="I14" s="99"/>
-      <c r="J14" s="99"/>
-      <c r="K14" s="99"/>
-      <c r="L14" s="99"/>
-      <c r="M14" s="100"/>
-    </row>
-    <row r="15" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="100"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="101"/>
+      <c r="E14" s="101"/>
+      <c r="F14" s="101"/>
+      <c r="G14" s="101"/>
+      <c r="H14" s="101"/>
+      <c r="I14" s="101"/>
+      <c r="J14" s="101"/>
+      <c r="K14" s="101"/>
+      <c r="L14" s="101"/>
+      <c r="M14" s="102"/>
+    </row>
+    <row r="15" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="35"/>
-      <c r="B15" s="98"/>
-      <c r="C15" s="99"/>
-      <c r="D15" s="99"/>
-      <c r="E15" s="99"/>
-      <c r="F15" s="99"/>
-      <c r="G15" s="99"/>
-      <c r="H15" s="99"/>
-      <c r="I15" s="99"/>
-      <c r="J15" s="99"/>
-      <c r="K15" s="99"/>
-      <c r="L15" s="99"/>
-      <c r="M15" s="100"/>
-    </row>
-    <row r="16" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B15" s="100"/>
+      <c r="C15" s="101"/>
+      <c r="D15" s="101"/>
+      <c r="E15" s="101"/>
+      <c r="F15" s="101"/>
+      <c r="G15" s="101"/>
+      <c r="H15" s="101"/>
+      <c r="I15" s="101"/>
+      <c r="J15" s="101"/>
+      <c r="K15" s="101"/>
+      <c r="L15" s="101"/>
+      <c r="M15" s="102"/>
+    </row>
+    <row r="16" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="35"/>
-      <c r="B16" s="98"/>
-      <c r="C16" s="99"/>
-      <c r="D16" s="99"/>
-      <c r="E16" s="99"/>
-      <c r="F16" s="99"/>
-      <c r="G16" s="99"/>
-      <c r="H16" s="99"/>
-      <c r="I16" s="99"/>
-      <c r="J16" s="99"/>
-      <c r="K16" s="99"/>
-      <c r="L16" s="99"/>
-      <c r="M16" s="100"/>
-    </row>
-    <row r="17" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="100"/>
+      <c r="C16" s="101"/>
+      <c r="D16" s="101"/>
+      <c r="E16" s="101"/>
+      <c r="F16" s="101"/>
+      <c r="G16" s="101"/>
+      <c r="H16" s="101"/>
+      <c r="I16" s="101"/>
+      <c r="J16" s="101"/>
+      <c r="K16" s="101"/>
+      <c r="L16" s="101"/>
+      <c r="M16" s="102"/>
+    </row>
+    <row r="17" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="35"/>
-      <c r="B17" s="98"/>
-      <c r="C17" s="99"/>
-      <c r="D17" s="99"/>
-      <c r="E17" s="99"/>
-      <c r="F17" s="99"/>
-      <c r="G17" s="99"/>
-      <c r="H17" s="99"/>
-      <c r="I17" s="99"/>
-      <c r="J17" s="99"/>
-      <c r="K17" s="99"/>
-      <c r="L17" s="99"/>
-      <c r="M17" s="100"/>
-    </row>
-    <row r="18" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B17" s="100"/>
+      <c r="C17" s="101"/>
+      <c r="D17" s="101"/>
+      <c r="E17" s="101"/>
+      <c r="F17" s="101"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="101"/>
+      <c r="I17" s="101"/>
+      <c r="J17" s="101"/>
+      <c r="K17" s="101"/>
+      <c r="L17" s="101"/>
+      <c r="M17" s="102"/>
+    </row>
+    <row r="18" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="35"/>
-      <c r="B18" s="98"/>
-      <c r="C18" s="99"/>
-      <c r="D18" s="99"/>
-      <c r="E18" s="99"/>
-      <c r="F18" s="99"/>
-      <c r="G18" s="99"/>
-      <c r="H18" s="99"/>
-      <c r="I18" s="99"/>
-      <c r="J18" s="99"/>
-      <c r="K18" s="99"/>
-      <c r="L18" s="99"/>
-      <c r="M18" s="100"/>
-    </row>
-    <row r="19" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="100"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="101"/>
+      <c r="E18" s="101"/>
+      <c r="F18" s="101"/>
+      <c r="G18" s="101"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="101"/>
+      <c r="J18" s="101"/>
+      <c r="K18" s="101"/>
+      <c r="L18" s="101"/>
+      <c r="M18" s="102"/>
+    </row>
+    <row r="19" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="35"/>
-      <c r="B19" s="98"/>
-      <c r="C19" s="99"/>
-      <c r="D19" s="99"/>
-      <c r="E19" s="99"/>
-      <c r="F19" s="99"/>
-      <c r="G19" s="99"/>
-      <c r="H19" s="99"/>
-      <c r="I19" s="99"/>
-      <c r="J19" s="99"/>
-      <c r="K19" s="99"/>
-      <c r="L19" s="99"/>
-      <c r="M19" s="100"/>
-    </row>
-    <row r="20" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B19" s="100"/>
+      <c r="C19" s="101"/>
+      <c r="D19" s="101"/>
+      <c r="E19" s="101"/>
+      <c r="F19" s="101"/>
+      <c r="G19" s="101"/>
+      <c r="H19" s="101"/>
+      <c r="I19" s="101"/>
+      <c r="J19" s="101"/>
+      <c r="K19" s="101"/>
+      <c r="L19" s="101"/>
+      <c r="M19" s="102"/>
+    </row>
+    <row r="20" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="35"/>
-      <c r="B20" s="98"/>
-      <c r="C20" s="99"/>
-      <c r="D20" s="99"/>
-      <c r="E20" s="99"/>
-      <c r="F20" s="99"/>
-      <c r="G20" s="99"/>
-      <c r="H20" s="99"/>
-      <c r="I20" s="99"/>
-      <c r="J20" s="99"/>
-      <c r="K20" s="99"/>
-      <c r="L20" s="99"/>
-      <c r="M20" s="100"/>
-    </row>
-    <row r="21" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B20" s="100"/>
+      <c r="C20" s="101"/>
+      <c r="D20" s="101"/>
+      <c r="E20" s="101"/>
+      <c r="F20" s="101"/>
+      <c r="G20" s="101"/>
+      <c r="H20" s="101"/>
+      <c r="I20" s="101"/>
+      <c r="J20" s="101"/>
+      <c r="K20" s="101"/>
+      <c r="L20" s="101"/>
+      <c r="M20" s="102"/>
+    </row>
+    <row r="21" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="35"/>
-      <c r="B21" s="98"/>
-      <c r="C21" s="99"/>
-      <c r="D21" s="99"/>
-      <c r="E21" s="99"/>
-      <c r="F21" s="99"/>
-      <c r="G21" s="99"/>
-      <c r="H21" s="99"/>
-      <c r="I21" s="99"/>
-      <c r="J21" s="99"/>
-      <c r="K21" s="99"/>
-      <c r="L21" s="99"/>
-      <c r="M21" s="100"/>
-    </row>
-    <row r="22" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B21" s="100"/>
+      <c r="C21" s="101"/>
+      <c r="D21" s="101"/>
+      <c r="E21" s="101"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="101"/>
+      <c r="H21" s="101"/>
+      <c r="I21" s="101"/>
+      <c r="J21" s="101"/>
+      <c r="K21" s="101"/>
+      <c r="L21" s="101"/>
+      <c r="M21" s="102"/>
+    </row>
+    <row r="22" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="35"/>
-      <c r="B22" s="98"/>
-      <c r="C22" s="99"/>
-      <c r="D22" s="99"/>
-      <c r="E22" s="99"/>
-      <c r="F22" s="99"/>
-      <c r="G22" s="99"/>
-      <c r="H22" s="99"/>
-      <c r="I22" s="99"/>
-      <c r="J22" s="99"/>
-      <c r="K22" s="99"/>
-      <c r="L22" s="99"/>
-      <c r="M22" s="100"/>
-    </row>
-    <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B22" s="100"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="101"/>
+      <c r="E22" s="101"/>
+      <c r="F22" s="101"/>
+      <c r="G22" s="101"/>
+      <c r="H22" s="101"/>
+      <c r="I22" s="101"/>
+      <c r="J22" s="101"/>
+      <c r="K22" s="101"/>
+      <c r="L22" s="101"/>
+      <c r="M22" s="102"/>
+    </row>
+    <row r="23" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="35"/>
-      <c r="B23" s="98"/>
-      <c r="C23" s="99"/>
-      <c r="D23" s="99"/>
-      <c r="E23" s="99"/>
-      <c r="F23" s="99"/>
-      <c r="G23" s="99"/>
-      <c r="H23" s="99"/>
-      <c r="I23" s="99"/>
-      <c r="J23" s="99"/>
-      <c r="K23" s="99"/>
-      <c r="L23" s="99"/>
-      <c r="M23" s="100"/>
-    </row>
-    <row r="24" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B23" s="100"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="101"/>
+      <c r="E23" s="101"/>
+      <c r="F23" s="101"/>
+      <c r="G23" s="101"/>
+      <c r="H23" s="101"/>
+      <c r="I23" s="101"/>
+      <c r="J23" s="101"/>
+      <c r="K23" s="101"/>
+      <c r="L23" s="101"/>
+      <c r="M23" s="102"/>
+    </row>
+    <row r="24" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="35"/>
-      <c r="B24" s="98"/>
-      <c r="C24" s="99"/>
-      <c r="D24" s="99"/>
-      <c r="E24" s="99"/>
-      <c r="F24" s="99"/>
-      <c r="G24" s="99"/>
-      <c r="H24" s="99"/>
-      <c r="I24" s="99"/>
-      <c r="J24" s="99"/>
-      <c r="K24" s="99"/>
-      <c r="L24" s="99"/>
-      <c r="M24" s="100"/>
-    </row>
-    <row r="25" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B24" s="100"/>
+      <c r="C24" s="101"/>
+      <c r="D24" s="101"/>
+      <c r="E24" s="101"/>
+      <c r="F24" s="101"/>
+      <c r="G24" s="101"/>
+      <c r="H24" s="101"/>
+      <c r="I24" s="101"/>
+      <c r="J24" s="101"/>
+      <c r="K24" s="101"/>
+      <c r="L24" s="101"/>
+      <c r="M24" s="102"/>
+    </row>
+    <row r="25" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="35"/>
-      <c r="B25" s="98"/>
-      <c r="C25" s="99"/>
-      <c r="D25" s="99"/>
-      <c r="E25" s="99"/>
-      <c r="F25" s="99"/>
-      <c r="G25" s="99"/>
-      <c r="H25" s="99"/>
-      <c r="I25" s="99"/>
-      <c r="J25" s="99"/>
-      <c r="K25" s="99"/>
-      <c r="L25" s="99"/>
-      <c r="M25" s="100"/>
-    </row>
-    <row r="26" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B25" s="100"/>
+      <c r="C25" s="101"/>
+      <c r="D25" s="101"/>
+      <c r="E25" s="101"/>
+      <c r="F25" s="101"/>
+      <c r="G25" s="101"/>
+      <c r="H25" s="101"/>
+      <c r="I25" s="101"/>
+      <c r="J25" s="101"/>
+      <c r="K25" s="101"/>
+      <c r="L25" s="101"/>
+      <c r="M25" s="102"/>
+    </row>
+    <row r="26" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="35"/>
-      <c r="B26" s="98"/>
-      <c r="C26" s="99"/>
-      <c r="D26" s="99"/>
-      <c r="E26" s="99"/>
-      <c r="F26" s="99"/>
-      <c r="G26" s="99"/>
-      <c r="H26" s="99"/>
-      <c r="I26" s="99"/>
-      <c r="J26" s="99"/>
-      <c r="K26" s="99"/>
-      <c r="L26" s="99"/>
-      <c r="M26" s="100"/>
-    </row>
-    <row r="27" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B26" s="100"/>
+      <c r="C26" s="101"/>
+      <c r="D26" s="101"/>
+      <c r="E26" s="101"/>
+      <c r="F26" s="101"/>
+      <c r="G26" s="101"/>
+      <c r="H26" s="101"/>
+      <c r="I26" s="101"/>
+      <c r="J26" s="101"/>
+      <c r="K26" s="101"/>
+      <c r="L26" s="101"/>
+      <c r="M26" s="102"/>
+    </row>
+    <row r="27" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="35"/>
-      <c r="B27" s="98"/>
-      <c r="C27" s="99"/>
-      <c r="D27" s="99"/>
-      <c r="E27" s="99"/>
-      <c r="F27" s="99"/>
-      <c r="G27" s="99"/>
-      <c r="H27" s="99"/>
-      <c r="I27" s="99"/>
-      <c r="J27" s="99"/>
-      <c r="K27" s="99"/>
-      <c r="L27" s="99"/>
-      <c r="M27" s="100"/>
-    </row>
-    <row r="28" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B27" s="100"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="101"/>
+      <c r="E27" s="101"/>
+      <c r="F27" s="101"/>
+      <c r="G27" s="101"/>
+      <c r="H27" s="101"/>
+      <c r="I27" s="101"/>
+      <c r="J27" s="101"/>
+      <c r="K27" s="101"/>
+      <c r="L27" s="101"/>
+      <c r="M27" s="102"/>
+    </row>
+    <row r="28" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="35"/>
-      <c r="B28" s="98"/>
-      <c r="C28" s="99"/>
-      <c r="D28" s="99"/>
-      <c r="E28" s="99"/>
-      <c r="F28" s="99"/>
-      <c r="G28" s="99"/>
-      <c r="H28" s="99"/>
-      <c r="I28" s="99"/>
-      <c r="J28" s="99"/>
-      <c r="K28" s="99"/>
-      <c r="L28" s="99"/>
-      <c r="M28" s="100"/>
-    </row>
-    <row r="29" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B28" s="100"/>
+      <c r="C28" s="101"/>
+      <c r="D28" s="101"/>
+      <c r="E28" s="101"/>
+      <c r="F28" s="101"/>
+      <c r="G28" s="101"/>
+      <c r="H28" s="101"/>
+      <c r="I28" s="101"/>
+      <c r="J28" s="101"/>
+      <c r="K28" s="101"/>
+      <c r="L28" s="101"/>
+      <c r="M28" s="102"/>
+    </row>
+    <row r="29" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="35"/>
-      <c r="B29" s="98"/>
-      <c r="C29" s="99"/>
-      <c r="D29" s="99"/>
-      <c r="E29" s="99"/>
-      <c r="F29" s="99"/>
-      <c r="G29" s="99"/>
-      <c r="H29" s="99"/>
-      <c r="I29" s="99"/>
-      <c r="J29" s="99"/>
-      <c r="K29" s="99"/>
-      <c r="L29" s="99"/>
-      <c r="M29" s="100"/>
-    </row>
-    <row r="30" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B29" s="100"/>
+      <c r="C29" s="101"/>
+      <c r="D29" s="101"/>
+      <c r="E29" s="101"/>
+      <c r="F29" s="101"/>
+      <c r="G29" s="101"/>
+      <c r="H29" s="101"/>
+      <c r="I29" s="101"/>
+      <c r="J29" s="101"/>
+      <c r="K29" s="101"/>
+      <c r="L29" s="101"/>
+      <c r="M29" s="102"/>
+    </row>
+    <row r="30" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="35"/>
-      <c r="B30" s="98"/>
-      <c r="C30" s="99"/>
-      <c r="D30" s="99"/>
-      <c r="E30" s="99"/>
-      <c r="F30" s="99"/>
-      <c r="G30" s="99"/>
-      <c r="H30" s="99"/>
-      <c r="I30" s="99"/>
-      <c r="J30" s="99"/>
-      <c r="K30" s="99"/>
-      <c r="L30" s="99"/>
-      <c r="M30" s="100"/>
-    </row>
-    <row r="31" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B30" s="100"/>
+      <c r="C30" s="101"/>
+      <c r="D30" s="101"/>
+      <c r="E30" s="101"/>
+      <c r="F30" s="101"/>
+      <c r="G30" s="101"/>
+      <c r="H30" s="101"/>
+      <c r="I30" s="101"/>
+      <c r="J30" s="101"/>
+      <c r="K30" s="101"/>
+      <c r="L30" s="101"/>
+      <c r="M30" s="102"/>
+    </row>
+    <row r="31" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="35"/>
-      <c r="B31" s="98"/>
-      <c r="C31" s="99"/>
-      <c r="D31" s="99"/>
-      <c r="E31" s="99"/>
-      <c r="F31" s="99"/>
-      <c r="G31" s="99"/>
-      <c r="H31" s="99"/>
-      <c r="I31" s="99"/>
-      <c r="J31" s="99"/>
-      <c r="K31" s="99"/>
-      <c r="L31" s="99"/>
-      <c r="M31" s="100"/>
-    </row>
-    <row r="32" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B31" s="100"/>
+      <c r="C31" s="101"/>
+      <c r="D31" s="101"/>
+      <c r="E31" s="101"/>
+      <c r="F31" s="101"/>
+      <c r="G31" s="101"/>
+      <c r="H31" s="101"/>
+      <c r="I31" s="101"/>
+      <c r="J31" s="101"/>
+      <c r="K31" s="101"/>
+      <c r="L31" s="101"/>
+      <c r="M31" s="102"/>
+    </row>
+    <row r="32" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="35"/>
-      <c r="B32" s="98"/>
-      <c r="C32" s="99"/>
-      <c r="D32" s="99"/>
-      <c r="E32" s="99"/>
-      <c r="F32" s="99"/>
-      <c r="G32" s="99"/>
-      <c r="H32" s="99"/>
-      <c r="I32" s="99"/>
-      <c r="J32" s="99"/>
-      <c r="K32" s="99"/>
-      <c r="L32" s="99"/>
-      <c r="M32" s="100"/>
-    </row>
-    <row r="33" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B32" s="100"/>
+      <c r="C32" s="101"/>
+      <c r="D32" s="101"/>
+      <c r="E32" s="101"/>
+      <c r="F32" s="101"/>
+      <c r="G32" s="101"/>
+      <c r="H32" s="101"/>
+      <c r="I32" s="101"/>
+      <c r="J32" s="101"/>
+      <c r="K32" s="101"/>
+      <c r="L32" s="101"/>
+      <c r="M32" s="102"/>
+    </row>
+    <row r="33" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="35"/>
-      <c r="B33" s="98"/>
-      <c r="C33" s="99"/>
-      <c r="D33" s="99"/>
-      <c r="E33" s="99"/>
-      <c r="F33" s="99"/>
-      <c r="G33" s="99"/>
-      <c r="H33" s="99"/>
-      <c r="I33" s="99"/>
-      <c r="J33" s="99"/>
-      <c r="K33" s="99"/>
-      <c r="L33" s="99"/>
-      <c r="M33" s="100"/>
-    </row>
-    <row r="34" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B33" s="100"/>
+      <c r="C33" s="101"/>
+      <c r="D33" s="101"/>
+      <c r="E33" s="101"/>
+      <c r="F33" s="101"/>
+      <c r="G33" s="101"/>
+      <c r="H33" s="101"/>
+      <c r="I33" s="101"/>
+      <c r="J33" s="101"/>
+      <c r="K33" s="101"/>
+      <c r="L33" s="101"/>
+      <c r="M33" s="102"/>
+    </row>
+    <row r="34" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="35"/>
-      <c r="B34" s="98"/>
-      <c r="C34" s="99"/>
-      <c r="D34" s="99"/>
-      <c r="E34" s="99"/>
-      <c r="F34" s="99"/>
-      <c r="G34" s="99"/>
-      <c r="H34" s="99"/>
-      <c r="I34" s="99"/>
-      <c r="J34" s="99"/>
-      <c r="K34" s="99"/>
-      <c r="L34" s="99"/>
-      <c r="M34" s="100"/>
-    </row>
-    <row r="35" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B34" s="100"/>
+      <c r="C34" s="101"/>
+      <c r="D34" s="101"/>
+      <c r="E34" s="101"/>
+      <c r="F34" s="101"/>
+      <c r="G34" s="101"/>
+      <c r="H34" s="101"/>
+      <c r="I34" s="101"/>
+      <c r="J34" s="101"/>
+      <c r="K34" s="101"/>
+      <c r="L34" s="101"/>
+      <c r="M34" s="102"/>
+    </row>
+    <row r="35" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="35"/>
-      <c r="B35" s="98"/>
-      <c r="C35" s="99"/>
-      <c r="D35" s="99"/>
-      <c r="E35" s="99"/>
-      <c r="F35" s="99"/>
-      <c r="G35" s="99"/>
-      <c r="H35" s="99"/>
-      <c r="I35" s="99"/>
-      <c r="J35" s="99"/>
-      <c r="K35" s="99"/>
-      <c r="L35" s="99"/>
-      <c r="M35" s="100"/>
-    </row>
-    <row r="36" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B35" s="100"/>
+      <c r="C35" s="101"/>
+      <c r="D35" s="101"/>
+      <c r="E35" s="101"/>
+      <c r="F35" s="101"/>
+      <c r="G35" s="101"/>
+      <c r="H35" s="101"/>
+      <c r="I35" s="101"/>
+      <c r="J35" s="101"/>
+      <c r="K35" s="101"/>
+      <c r="L35" s="101"/>
+      <c r="M35" s="102"/>
+    </row>
+    <row r="36" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="35"/>
-      <c r="B36" s="98"/>
-      <c r="C36" s="99"/>
-      <c r="D36" s="99"/>
-      <c r="E36" s="99"/>
-      <c r="F36" s="99"/>
-      <c r="G36" s="99"/>
-      <c r="H36" s="99"/>
-      <c r="I36" s="99"/>
-      <c r="J36" s="99"/>
-      <c r="K36" s="99"/>
-      <c r="L36" s="99"/>
-      <c r="M36" s="100"/>
-    </row>
-    <row r="37" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B36" s="100"/>
+      <c r="C36" s="101"/>
+      <c r="D36" s="101"/>
+      <c r="E36" s="101"/>
+      <c r="F36" s="101"/>
+      <c r="G36" s="101"/>
+      <c r="H36" s="101"/>
+      <c r="I36" s="101"/>
+      <c r="J36" s="101"/>
+      <c r="K36" s="101"/>
+      <c r="L36" s="101"/>
+      <c r="M36" s="102"/>
+    </row>
+    <row r="37" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="35"/>
-      <c r="B37" s="98"/>
-      <c r="C37" s="99"/>
-      <c r="D37" s="99"/>
-      <c r="E37" s="99"/>
-      <c r="F37" s="99"/>
-      <c r="G37" s="99"/>
-      <c r="H37" s="99"/>
-      <c r="I37" s="99"/>
-      <c r="J37" s="99"/>
-      <c r="K37" s="99"/>
-      <c r="L37" s="99"/>
-      <c r="M37" s="100"/>
-    </row>
-    <row r="38" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B37" s="100"/>
+      <c r="C37" s="101"/>
+      <c r="D37" s="101"/>
+      <c r="E37" s="101"/>
+      <c r="F37" s="101"/>
+      <c r="G37" s="101"/>
+      <c r="H37" s="101"/>
+      <c r="I37" s="101"/>
+      <c r="J37" s="101"/>
+      <c r="K37" s="101"/>
+      <c r="L37" s="101"/>
+      <c r="M37" s="102"/>
+    </row>
+    <row r="38" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="35"/>
-      <c r="B38" s="98"/>
-      <c r="C38" s="99"/>
-      <c r="D38" s="99"/>
-      <c r="E38" s="99"/>
-      <c r="F38" s="99"/>
-      <c r="G38" s="99"/>
-      <c r="H38" s="99"/>
-      <c r="I38" s="99"/>
-      <c r="J38" s="99"/>
-      <c r="K38" s="99"/>
-      <c r="L38" s="99"/>
-      <c r="M38" s="100"/>
-    </row>
-    <row r="39" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B38" s="100"/>
+      <c r="C38" s="101"/>
+      <c r="D38" s="101"/>
+      <c r="E38" s="101"/>
+      <c r="F38" s="101"/>
+      <c r="G38" s="101"/>
+      <c r="H38" s="101"/>
+      <c r="I38" s="101"/>
+      <c r="J38" s="101"/>
+      <c r="K38" s="101"/>
+      <c r="L38" s="101"/>
+      <c r="M38" s="102"/>
+    </row>
+    <row r="39" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="35"/>
-      <c r="B39" s="101"/>
-      <c r="C39" s="102"/>
-      <c r="D39" s="102"/>
-      <c r="E39" s="102"/>
-      <c r="F39" s="102"/>
-      <c r="G39" s="102"/>
-      <c r="H39" s="102"/>
-      <c r="I39" s="102"/>
-      <c r="J39" s="102"/>
-      <c r="K39" s="102"/>
-      <c r="L39" s="102"/>
-      <c r="M39" s="103"/>
+      <c r="B39" s="103"/>
+      <c r="C39" s="104"/>
+      <c r="D39" s="104"/>
+      <c r="E39" s="104"/>
+      <c r="F39" s="104"/>
+      <c r="G39" s="104"/>
+      <c r="H39" s="104"/>
+      <c r="I39" s="104"/>
+      <c r="J39" s="104"/>
+      <c r="K39" s="104"/>
+      <c r="L39" s="104"/>
+      <c r="M39" s="105"/>
     </row>
     <row r="40" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="35"/>
@@ -53299,12 +53299,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="90750662-e876-4027-87c5-760b0ce6cf5c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c036ba9-6adb-4bb7-998f-df2d2059af4e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -53554,22 +53558,28 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="90750662-e876-4027-87c5-760b0ce6cf5c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c036ba9-6adb-4bb7-998f-df2d2059af4e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0A3F0B4-9A99-4E66-9809-E917735194F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7AB8550-DBC3-48E6-A43C-536AC3D2748B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="7c036ba9-6adb-4bb7-998f-df2d2059af4e"/>
+    <ds:schemaRef ds:uri="90750662-e876-4027-87c5-760b0ce6cf5c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -53595,19 +53605,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7AB8550-DBC3-48E6-A43C-536AC3D2748B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0A3F0B4-9A99-4E66-9809-E917735194F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="7c036ba9-6adb-4bb7-998f-df2d2059af4e"/>
-    <ds:schemaRef ds:uri="90750662-e876-4027-87c5-760b0ce6cf5c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>